<commit_message>
투자 대시보드 2026-10-13 18:25
</commit_message>
<xml_diff>
--- a/technicals/exports/2026-10-12.xlsx
+++ b/technicals/exports/2026-10-12.xlsx
@@ -142,7 +142,7 @@
       </ns0:c>
       <ns0:c r="F2" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 의약품과 치료제를 연구·개발·제조·판매하는 연구 중심 바이오 제약 기업.</ns0:t>
+          <ns0:t>전 세계에서 의약품·치료제를 연구·개발·제조·판매하는 연구 중심 바이오 제약 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G2">
@@ -221,7 +221,7 @@
       </ns0:c>
       <ns0:c r="F3" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 건설·엔지니어링 구조물·운송 시장에 인프라 관련 제품과 솔루션을 제공한다.</ns0:t>
+          <ns0:t>미국 건설·엔지니어링 구조물·운송 시장에 인프라 제품과 솔루션을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G3">
@@ -300,7 +300,7 @@
       </ns0:c>
       <ns0:c r="F4" t="inlineStr">
         <ns0:is>
-          <ns0:t>계열사를 통해 미국 펀드, 기관, 개인 및 고액자산가에게 투자관리·자문 서비스를 제공.</ns0:t>
+          <ns0:t>계열사를 통해 미국 펀드·기관·개인·고액자산가에게 투자관리·자문 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G4">
@@ -379,7 +379,7 @@
       </ns0:c>
       <ns0:c r="F5" t="inlineStr">
         <ns0:is>
-          <ns0:t>디지털 제품의 고객 행동을 분석하는 AI 플랫폼과 실시간 분석·세션 재생 도구를 제공.</ns0:t>
+          <ns0:t>디지털 제품의 고객 행동 분석용 AI 플랫폼과 실시간 분석·세션 재생 도구를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G5">
@@ -537,7 +537,7 @@
       </ns0:c>
       <ns0:c r="F7" t="inlineStr">
         <ns0:is>
-          <ns0:t>다발성경화증, 척수성 근위축증 등 치료제를 연구·개발·제조·공급하는 기업.</ns0:t>
+          <ns0:t>다발성경화증·척수성 근위축증 등 치료제를 연구·개발·제조·공급하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G7">
@@ -616,7 +616,7 @@
       </ns0:c>
       <ns0:c r="F8" t="inlineStr">
         <ns0:is>
-          <ns0:t>기업과의 합병, 주식 교환, 자산 인수 등 사업 결합을 추진하는 기업.</ns0:t>
+          <ns0:t>합병·주식 교환·자산 인수 등 기업과의 사업 결합을 추진하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G8">
@@ -692,7 +692,7 @@
       </ns0:c>
       <ns0:c r="F9" t="inlineStr">
         <ns0:is>
-          <ns0:t>다양한 규모의 조직이 장소와 기기에 관계없이 콘텐츠를 관리하는 클라우드 플랫폼 제공.</ns0:t>
+          <ns0:t>다양한 규모의 조직이 장소·기기에 관계없이 콘텐츠를 관리하는 클라우드 플랫폼 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G9">
@@ -771,7 +771,7 @@
       </ns0:c>
       <ns0:c r="F10" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 선박 보유·용선, 액화석유가스 운송 및 통합 배송 서비스를 제공.</ns0:t>
+          <ns0:t>전 세계에서 선박 보유·용선, 액화석유가스 운송 및 통합 배송 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G10">
@@ -1008,7 +1008,7 @@
       </ns0:c>
       <ns0:c r="F13" t="inlineStr">
         <ns0:is>
-          <ns0:t>벨기에 해운 기업으로 해운·수소 인프라·수소 산업 부문을 운영하며 저탄소·무탄소 선박을 설계·건조·운영.</ns0:t>
+          <ns0:t>해운·수소 인프라·수소 산업을 운영하며 저탄소·무탄소 선박을 설계·건조·운영하는 벨기에 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G13">
@@ -1087,7 +1087,7 @@
       </ns0:c>
       <ns0:c r="F14" t="inlineStr">
         <ns0:is>
-          <ns0:t>기업·공공부문 등에 컴퓨터 시스템과 데이터센터를 포함한 다양한 IT 솔루션을 제공하는 기업.</ns0:t>
+          <ns0:t>기업·공공부문에 컴퓨터 시스템·데이터센터 등 다양한 IT 솔루션을 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G14">
@@ -1166,7 +1166,7 @@
       </ns0:c>
       <ns0:c r="F15" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 직업건강센터와 사업장 내 진료소 등을 통해 직업건강 및 고용주·소비자 건강 서비스를 제공.</ns0:t>
+          <ns0:t>미국에서 직업건강센터와 사업장 내 진료소를 통해 직업건강 및 고용주·소비자 건강 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G15">
@@ -1245,7 +1245,7 @@
       </ns0:c>
       <ns0:c r="F16" t="inlineStr">
         <ns0:is>
-          <ns0:t>컨테이너선과 건화물선을 보유·운영하며 해상 운송 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>컨테이너선·건화물선을 보유·운영하며 해상 운송 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G16">
@@ -1324,7 +1324,7 @@
       </ns0:c>
       <ns0:c r="F17" t="inlineStr">
         <ns0:is>
-          <ns0:t>클라우드 애플리케이션용 관측·보안 플랫폼과 인프라·성능 모니터링, 로그 관리 등을 제공.</ns0:t>
+          <ns0:t>클라우드 앱 관측·보안 플랫폼과 인프라·성능 모니터링, 로그 관리 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G17">
@@ -1403,7 +1403,7 @@
       </ns0:c>
       <ns0:c r="F18" t="inlineStr">
         <ns0:is>
-          <ns0:t>자회사를 통해 원유 운반선을 소유·운영하며 기술 관리 서비스도 제공하는 기업.</ns0:t>
+          <ns0:t>자회사를 통해 원유 운반선을 소유·운영하고 기술 관리 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G18">
@@ -1482,7 +1482,7 @@
       </ns0:c>
       <ns0:c r="F19" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 독립 에너지 기업으로 정유·재생에너지·마케팅·윤활유·미드스트림 사업과 연료 생산·판매를 수행.</ns0:t>
+          <ns0:t>미국 독립 에너지 기업으로 정유·재생에너지·윤활유·미드스트림 사업과 연료 생산·판매 수행.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G19">
@@ -1561,7 +1561,7 @@
       </ns0:c>
       <ns0:c r="F20" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 사이버보안·AI 등 분야 기업과의 합병·인수를 추진하는 기업.</ns0:t>
+          <ns0:t>주요 영업활동 없이 사이버보안·AI 등 분야 기업과의 합병·인수를 추진.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G20">
@@ -1637,7 +1637,7 @@
       </ns0:c>
       <ns0:c r="F21" t="inlineStr">
         <ns0:is>
-          <ns0:t>디지털 기업의 복잡한 디지털 환경을 위한 AI 기반 관측성 플랫폼을 제공하는 기업.</ns0:t>
+          <ns0:t>기업의 복잡한 디지털 환경을 위한 AI 기반 관측성 플랫폼 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G21">
@@ -1874,7 +1874,7 @@
       </ns0:c>
       <ns0:c r="F24" t="inlineStr">
         <ns0:is>
-          <ns0:t>멀티클라우드 애플리케이션 보안·전송 솔루션과 앱 배포·보안·운영용 분산 클라우드 서비스를 제공한다.</ns0:t>
+          <ns0:t>멀티클라우드 앱 보안·전송 솔루션과 앱 배포·보안·운영을 위한 분산 클라우드 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G24">
@@ -1953,7 +1953,7 @@
       </ns0:c>
       <ns0:c r="F25" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 의료용 의류, 신발 등 생활용품을 소비자에게 직접 판매하는 기업.</ns0:t>
+          <ns0:t>미국과 해외에서 의료용 의류·신발 등 생활용품을 소비자에게 직접 판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G25">
@@ -2032,7 +2032,7 @@
       </ns0:c>
       <ns0:c r="F26" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 초대형 원유운반선, 수에즈막스, LR2·아프라막스 등 원유·석유제품 운반선을 보유·운영.</ns0:t>
+          <ns0:t>전 세계에서 초대형·수에즈막스·LR2·아프라막스 원유·석유제품 운반선 보유·운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G26">
@@ -2111,7 +2111,7 @@
       </ns0:c>
       <ns0:c r="F27" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 사이버보안 및 네트워크·보안 통합 솔루션을 제공하는 기업.</ns0:t>
+          <ns0:t>전 세계에 사이버보안과 네트워크·보안 통합 솔루션을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G27">
@@ -2269,7 +2269,7 @@
       </ns0:c>
       <ns0:c r="F29" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·호주·유럽의 매장과 온라인에서 게임, 수집품, 엔터테인먼트 제품을 판매하는 기업.</ns0:t>
+          <ns0:t>미국·호주·유럽의 매장과 온라인에서 게임·수집품·엔터테인먼트 제품을 판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G29">
@@ -2348,7 +2348,7 @@
       </ns0:c>
       <ns0:c r="F30" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 및 해외에서 에너지 서비스를 제공하며 전력·천연가스 재판매와 재생에너지 사업을 영위.</ns0:t>
+          <ns0:t>미국 및 해외에서 전력·천연가스 재판매와 재생에너지 등 에너지 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G30">
@@ -2427,7 +2427,7 @@
       </ns0:c>
       <ns0:c r="F31" t="inlineStr">
         <ns0:is>
-          <ns0:t>소프트웨어 개발 전 과정을 지원하는 통합 DevSecOps 플랫폼 GitLab을 제공하는 기업.</ns0:t>
+          <ns0:t>소프트웨어 개발 전 과정을 지원하는 통합 DevSecOps 플랫폼 GitLab을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G31">
@@ -2506,7 +2506,7 @@
       </ns0:c>
       <ns0:c r="F32" t="inlineStr">
         <ns0:is>
-          <ns0:t>혈장·혈액센터·병원 부문의 의료기술 기업으로 자동 혈장 채취 시스템과 헌혈자 관리 소프트웨어 등을 제공.</ns0:t>
+          <ns0:t>혈장·혈액센터·병원용 의료기술 기업으로 자동 혈장 채취 시스템과 헌혈자 관리 소프트웨어 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G32">
@@ -2664,7 +2664,7 @@
       </ns0:c>
       <ns0:c r="F34" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다·영국에서 수집용·자동차 애호가용 차량 보험을 제공하며 보험·마켓플레이스 부문을 운영.</ns0:t>
+          <ns0:t>미국·캐나다·영국에서 수집용·자동차 애호가용 차량 보험과 마켓플레이스 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G34">
@@ -2743,7 +2743,7 @@
       </ns0:c>
       <ns0:c r="F35" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국과 해외에서 다양한 형태의 맞춤형 냉간 성형 강재를 제조·판매하는 회사.</ns0:t>
+          <ns0:t>중국과 해외에서 다양한 맞춤형 냉간 성형 강재를 제조·판매한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G35">
@@ -2822,7 +2822,7 @@
       </ns0:c>
       <ns0:c r="F36" t="inlineStr">
         <ns0:is>
-          <ns0:t>기술로 의료 제공을 확장·자동화하며 급성 부상·만성 통증·수술 후 재활 등 근골격계 관리 플랫폼을 개발하는 기업.</ns0:t>
+          <ns0:t>급성 부상·만성 통증·수술 후 재활 등 근골격계 관리를 위한 의료 자동화 플랫폼 개발 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G36">
@@ -2980,7 +2980,7 @@
       </ns0:c>
       <ns0:c r="F38" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 의료기관에 SaaS 애플리케이션과 의료 제공자 채용·신청·면허 검증 등 관리 도구를 제공.</ns0:t>
+          <ns0:t>미국 의료기관에 SaaS와 의료 제공자 채용·신청·면허 검증 관리 도구를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G38">
@@ -3059,7 +3059,7 @@
       </ns0:c>
       <ns0:c r="F39" t="inlineStr">
         <ns0:is>
-          <ns0:t>기술 기반 고객 경험 솔루션과 고객서비스·기술지원·백오피스 아웃소싱을 제공하는 기업.</ns0:t>
+          <ns0:t>기술 기반 고객 경험 솔루션과 고객서비스·기술지원·백오피스 아웃소싱을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G39">
@@ -3138,7 +3138,7 @@
       </ns0:c>
       <ns0:c r="F40" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·영국 등에서 핀테크 및 통신 솔루션을 제공하는 기업.</ns0:t>
+          <ns0:t>미국·영국 등에서 핀테크 및 통신 솔루션 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G40">
@@ -3217,7 +3217,7 @@
       </ns0:c>
       <ns0:c r="F41" t="inlineStr">
         <ns0:is>
-          <ns0:t>기업과의 합병, 주식 교환, 자산 인수 등 사업 결합을 추진하는 기업.</ns0:t>
+          <ns0:t>합병·주식 교환·자산 인수 등 사업 결합을 추진하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G41">
@@ -3293,7 +3293,7 @@
       </ns0:c>
       <ns0:c r="F42" t="inlineStr">
         <ns0:is>
-          <ns0:t>원유와 석유제품의 국제 해상 운송을 위해 원유선과 제품 운반선을 보유·운영하는 기업.</ns0:t>
+          <ns0:t>원유선과 석유제품 운반선을 보유·운영하며 원유·석유제품의 국제 해상 운송을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G42">
@@ -3372,7 +3372,7 @@
       </ns0:c>
       <ns0:c r="F43" t="inlineStr">
         <ns0:is>
-          <ns0:t>소셜 서비스와 통신 기술을 제공하며 소셜 라이브 스트리밍 플랫폼 Bigo Live를 운영한다.</ns0:t>
+          <ns0:t>소셜 서비스·통신 기술을 제공하고 소셜 라이브 스트리밍 플랫폼 Bigo Live를 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G43">
@@ -3451,7 +3451,7 @@
       </ns0:c>
       <ns0:c r="F44" t="inlineStr">
         <ns0:is>
-          <ns0:t>외식업용 플라스틱·종이·바이오폴리머·퇴비화 소재 일회용 용기와 포장재를 제조·유통하는 기업.</ns0:t>
+          <ns0:t>외식업용 플라스틱·종이·바이오폴리머·퇴비화 소재 일회용 용기와 포장재를 제조·유통.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G44">
@@ -3530,7 +3530,7 @@
       </ns0:c>
       <ns0:c r="F45" t="inlineStr">
         <ns0:is>
-          <ns0:t>맞춤형 선박을 활용한 해양 탐험과 육상 여행 체험을 전 세계에 제공하는 기업.</ns0:t>
+          <ns0:t>맞춤형 선박을 활용한 해양 탐험과 육상 여행 체험을 전 세계에 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G45">
@@ -3688,7 +3688,7 @@
       </ns0:c>
       <ns0:c r="F47" t="inlineStr">
         <ns0:is>
-          <ns0:t>버뮤다와 해외에서 이중선체 유조선을 보유·운영·용선하며 석유회사와 원유 거래업체에 서비스를 제공.</ns0:t>
+          <ns0:t>버뮤다와 해외에서 이중선체 유조선을 보유·운영·용선하며 석유회사·원유 거래업체에 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G47">
@@ -3846,7 +3846,7 @@
       </ns0:c>
       <ns0:c r="F49" t="inlineStr">
         <ns0:is>
-          <ns0:t>하이브리드·퍼블릭 클라우드 부문에서 데이터 인프라용 기업 소프트웨어·시스템·서비스를 개발하는 기업.</ns0:t>
+          <ns0:t>하이브리드·퍼블릭 클라우드의 데이터 인프라용 기업 소프트웨어·시스템·서비스를 개발.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G49">
@@ -4004,7 +4004,7 @@
       </ns0:c>
       <ns0:c r="F51" t="inlineStr">
         <ns0:is>
-          <ns0:t>자동차 금융·리스, 은행 및 금융서비스 산업용 기업 소프트웨어를 설계·개발·판매하는 회사.</ns0:t>
+          <ns0:t>자동차 금융·리스, 은행·금융서비스용 기업 소프트웨어를 설계·개발·판매하는 회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G51">
@@ -4083,7 +4083,7 @@
       </ns0:c>
       <ns0:c r="F52" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 싱글 사인온과 위험 기반 다중요소 인증 등 신원·접근 보안 서비스를 제공하는 회사.</ns0:t>
+          <ns0:t>미국과 해외에서 싱글 사인온, 위험 기반 다중요소 인증 등 신원·접근 보안 서비스를 제공하는 회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G52">
@@ -4162,7 +4162,7 @@
       </ns0:c>
       <ns0:c r="F53" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 온라인·전화·매장 및 제휴 채널을 통해 개인대출과 신용카드를 제공.</ns0:t>
+          <ns0:t>미국에서 온라인·전화·매장 및 제휴 채널을 통해 개인대출과 신용카드 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G53">
@@ -4241,7 +4241,7 @@
       </ns0:c>
       <ns0:c r="F54" t="inlineStr">
         <ns0:is>
-          <ns0:t>선불카드, 환자 비용 부담 지원, 디지털뱅킹, 생명과학 소프트웨어 및 통합 결제처리를 제공하는 회사.</ns0:t>
+          <ns0:t>선불카드, 환자 비용 지원, 디지털뱅킹, 생명과학 소프트웨어 및 통합 결제처리를 제공하는 회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G54">
@@ -4320,7 +4320,7 @@
       </ns0:c>
       <ns0:c r="F55" t="inlineStr">
         <ns0:is>
-          <ns0:t>브라질과 해외에서 석유·가스를 탐사·생산·판매하며 정유·운송·판매 사업을 운영한다.</ns0:t>
+          <ns0:t>브라질과 해외에서 석유·가스 탐사·생산·판매 및 정유·운송 사업을 운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G55">
@@ -4399,7 +4399,7 @@
       </ns0:c>
       <ns0:c r="F56" t="inlineStr">
         <ns0:is>
-          <ns0:t>브라질과 해외에서 석유·가스를 탐사·생산·판매하며 정유·운송·판매 사업을 운영한다.</ns0:t>
+          <ns0:t>브라질과 해외에서 석유·가스 탐사·생산·판매 및 정유·운송 사업을 운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G56">
@@ -4478,7 +4478,7 @@
       </ns0:c>
       <ns0:c r="F57" t="inlineStr">
         <ns0:is>
-          <ns0:t>암 치료 제품을 개발·상용화하는 바이오제약 기업으로 경구용 네라티닙인 NERLYNX를 제공.</ns0:t>
+          <ns0:t>암 치료제를 개발·상용화하는 바이오제약 기업으로 경구용 네라티닙 NERLYNX 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G57">
@@ -4557,7 +4557,7 @@
       </ns0:c>
       <ns0:c r="F58" t="inlineStr">
         <ns0:is>
-          <ns0:t>정보기관의 대테러 조사·작전을 지원하는 소프트웨어 플랫폼을 구축·배포하고 국방 솔루션 제공.</ns0:t>
+          <ns0:t>정보기관의 대테러 조사·작전을 지원하는 소프트웨어 플랫폼과 국방 솔루션을 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G58">
@@ -4715,7 +4715,7 @@
       </ns0:c>
       <ns0:c r="F60" t="inlineStr">
         <ns0:is>
-          <ns0:t>당좌·저축·정기예금과 개인·기업·농업·상업용 부동산·주택담보 대출 등 은행 서비스를 제공한다.</ns0:t>
+          <ns0:t>당좌·저축·정기예금과 개인·기업·농업·상업용 부동산·주택담보 대출 서비스를 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G60">
@@ -4873,7 +4873,7 @@
       </ns0:c>
       <ns0:c r="F62" t="inlineStr">
         <ns0:is>
-          <ns0:t>텍사스·뉴멕시코에서 석유·천연가스·천연가스액 자산을 인수·탐사·개발·생산.</ns0:t>
+          <ns0:t>텍사스·뉴멕시코에서 석유·천연가스·천연가스액 자산을 인수·탐사·개발·생산한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G62">
@@ -4952,7 +4952,7 @@
       </ns0:c>
       <ns0:c r="F63" t="inlineStr">
         <ns0:is>
-          <ns0:t>온라인 판매자와 소비자의 신뢰 관계 구축을 돕는 전자상거래 위험 분석 플랫폼을 개발·제공한다.</ns0:t>
+          <ns0:t>온라인 판매자와 소비자의 신뢰 구축을 돕는 전자상거래 위험 분석 플랫폼을 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G63">
@@ -5031,7 +5031,7 @@
       </ns0:c>
       <ns0:c r="F64" t="inlineStr">
         <ns0:is>
-          <ns0:t>세계 각지에서 통합 가스, 자원 개발·생산, 마케팅, 화학·제품, 재생에너지 사업을 운영한다.</ns0:t>
+          <ns0:t>전 세계에서 통합 가스, 자원 개발·생산, 마케팅, 화학·제품, 재생에너지 사업을 운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G64">
@@ -5110,7 +5110,7 @@
       </ns0:c>
       <ns0:c r="F65" t="inlineStr">
         <ns0:is>
-          <ns0:t>실질적인 영업활동 없이 합병, 주식 교환, 자산 인수 등 기업결합을 추진하는 회사.</ns0:t>
+          <ns0:t>실질적 영업활동 없이 합병·주식교환·자산인수 등 기업결합을 추진.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G65">
@@ -5186,7 +5186,7 @@
       </ns0:c>
       <ns0:c r="F66" t="inlineStr">
         <ns0:is>
-          <ns0:t>남아공 등에서 화학·에너지 사업을 운영하며 역청, 연료, 나프타, 윤활유, 액화석유가스 등을 공급한다.</ns0:t>
+          <ns0:t>남아공 등에서 화학·에너지 사업을 운영하며 역청·연료·나프타·윤활유·액화석유가스를 공급한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G66">
@@ -5265,7 +5265,7 @@
       </ns0:c>
       <ns0:c r="F67" t="inlineStr">
         <ns0:is>
-          <ns0:t>캐나다·미국 등에서 오일샌드, 석유 탐사·생산, 정유·판매 사업을 영위하는 종합 에너지 기업.</ns0:t>
+          <ns0:t>캐나다·미국 등에서 오일샌드, 석유 탐사·생산, 정유·판매 사업을 운영하는 종합 에너지 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G67">
@@ -5502,7 +5502,7 @@
       </ns0:c>
       <ns0:c r="F70" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 원유 해상운송과 해양 서비스를 제공하며 원유·정유제품 운반선을 보유·운영한다.</ns0:t>
+          <ns0:t>세계적으로 원유 해상운송·해양 서비스를 제공하며 원유·정유제품 운반선을 보유·운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G70">
@@ -5581,7 +5581,7 @@
       </ns0:c>
       <ns0:c r="F71" t="inlineStr">
         <ns0:is>
-          <ns0:t>석유업계에 해상 운송, 항해·기간 용선, 해상 선박 간 화물 이송 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>석유업계에 해상 운송·항해 및 기간 용선·해상 선박 간 화물 이송 서비스를 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G71">
@@ -5739,7 +5739,7 @@
       </ns0:c>
       <ns0:c r="F73" t="inlineStr">
         <ns0:is>
-          <ns0:t>실질적인 영업활동 없이 다른 기업과의 합병·주식교환·자산인수 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>실질적 영업활동 없이 합병·주식교환·자산인수 등 다른 기업과의 기업결합을 추진.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G73">
@@ -5815,7 +5815,7 @@
       </ns0:c>
       <ns0:c r="F74" t="inlineStr">
         <ns0:is>
-          <ns0:t>결제 승인·청산·정산 네트워크 VisaNet을 운영하고 신용·직불·선불카드 상품을 제공.</ns0:t>
+          <ns0:t>결제 승인·청산·정산 네트워크 VisaNet을 운영하고 신용·직불·선불카드 상품을 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G74">
@@ -5894,7 +5894,7 @@
       </ns0:c>
       <ns0:c r="F75" t="inlineStr">
         <ns0:is>
-          <ns0:t>파키스탄·우크라이나·카자흐스탄·방글라데시·우즈베키스탄에서 이동통신과 디지털 서비스를 제공.</ns0:t>
+          <ns0:t>파키스탄·우크라이나·카자흐스탄·방글라데시·우즈베키스탄에서 이동통신·디지털 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G75">
@@ -6131,7 +6131,7 @@
       </ns0:c>
       <ns0:c r="F78" t="inlineStr">
         <ns0:is>
-          <ns0:t>자회사 Win-Fung을 통해 말레이시아 등에서 유리섬유 강화 플라스틱 제품과 탱크·라이닝 제품을 제조·공급한다.</ns0:t>
+          <ns0:t>자회사 Win-Fung을 통해 말레이시아 등에서 유리섬유 강화 플라스틱·탱크·라이닝 제품을 제조·공급한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G78">
@@ -6210,7 +6210,7 @@
       </ns0:c>
       <ns0:c r="F79" t="inlineStr">
         <ns0:is>
-          <ns0:t>브라질에서 개방형 투자 플랫폼을 통해 증권·채권·펀드 등 금융상품과 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>브라질의 개방형 투자 플랫폼으로 증권·채권·펀드 등 금융상품과 서비스를 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G79">
@@ -6289,7 +6289,7 @@
       </ns0:c>
       <ns0:c r="F80" t="inlineStr">
         <ns0:is>
-          <ns0:t>이스라엘과 해외에서 컨테이너 해운과 문전·항만 간 운송 등 관련 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>이스라엘과 해외에서 컨테이너 해운 및 문전·항만 간 운송 서비스를 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G80">

</xml_diff>